<commit_message>
refine wizard FX guardrails, field visibility, and default report templates
</commit_message>
<xml_diff>
--- a/default_template/template_domestic.xlsx
+++ b/default_template/template_domestic.xlsx
@@ -10,7 +10,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="List" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'List'!$A$1:$F$62</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Report'!$A$1:$K$25</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -626,7 +629,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -642,7 +645,7 @@
     <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LEK Partners</t>
+          <t>KIOTI</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1284,9 @@
     <mergeCell ref="A61:B61"/>
     <mergeCell ref="B4:C4"/>
   </mergeCells>
+  <printOptions horizontalCentered="1" verticalCentered="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1289,7 +1294,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1310,7 +1315,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>LEK Partners</t>
+          <t>KIOTI</t>
         </is>
       </c>
     </row>
@@ -1721,6 +1726,8 @@
     <mergeCell ref="G23:I23"/>
     <mergeCell ref="A16:C16"/>
   </mergeCells>
+  <printOptions horizontalCentered="1" verticalCentered="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>